<commit_message>
fix(crm): update lead defaults to New Lead, 10-day credit, Person 1-6 reps, and full 55 product rate master
</commit_message>
<xml_diff>
--- a/KTA_Executive_Marketing_CRM_Master.xlsx
+++ b/KTA_Executive_Marketing_CRM_Master.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Client Accounts" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Warehouse Inventory &amp; QC" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignment Dispatch Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Rate Master" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,11 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; kg&quot;"/>
+    <numFmt numFmtId="166" formatCode="₹ #,##,##0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +83,37 @@
       <color rgb="00111827"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E2814"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001A1A1A"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -159,8 +190,26 @@
         <bgColor rgb="00BFA15F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E2814"/>
+        <bgColor rgb="001E2814"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002D3A1F"/>
+        <bgColor rgb="002D3A1F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAF6"/>
+        <bgColor rgb="00F8FAF6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -182,11 +231,25 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D8E2D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D8E2D6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D8E2D6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D8E2D6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -282,6 +345,42 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1356,7 +1455,6 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -1402,7 +1500,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
@@ -1410,7 +1507,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -3798,4 +3894,2007 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="68" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>KTA SPICES - PRODUCT MASTER &amp; COMMERCIAL RATE CARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Master SKU Price Reference: HSN Codes, Benchmark Rates &amp; Wholesale Packaging Specifications (55 Varieties)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>SKU Code</t>
+        </is>
+      </c>
+      <c r="B4" s="36" t="inlineStr">
+        <is>
+          <t>Product Variety Name</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>HSN Code</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Base Rate (₹/kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="36" t="inlineStr">
+        <is>
+          <t>Wholesale MOQ</t>
+        </is>
+      </c>
+      <c r="G4" s="36" t="inlineStr">
+        <is>
+          <t>Culinary Grade &amp; Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-001</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="inlineStr">
+        <is>
+          <t>Tellicherry Black Pepper (TGSEB Bold Whole)</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>09041140</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>720</v>
+      </c>
+      <c r="F5" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>Bold export-grade Tellicherry whole black peppercorns (4.75mm+). High aroma &amp; heat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-002</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>Single-Origin Black Pepper Powder (Cold-Milled)</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D6" s="43" t="inlineStr">
+        <is>
+          <t>09041200</t>
+        </is>
+      </c>
+      <c r="E6" s="44" t="n">
+        <v>750</v>
+      </c>
+      <c r="F6" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>Coarse &amp; fine chef-grade ground black pepper. Zero pinhead waste or fillers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-003</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="inlineStr">
+        <is>
+          <t>Decorticated White Pepper (Whole)</t>
+        </is>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D7" s="39" t="inlineStr">
+        <is>
+          <t>09041190</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F7" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G7" s="38" t="inlineStr">
+        <is>
+          <t>Naturally water-retted decorticated white peppercorns for continental dining.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-004</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>Fine Milled White Pepper Powder</t>
+        </is>
+      </c>
+      <c r="C8" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D8" s="43" t="inlineStr">
+        <is>
+          <t>09041200</t>
+        </is>
+      </c>
+      <c r="E8" s="44" t="n">
+        <v>1080</v>
+      </c>
+      <c r="F8" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G8" s="42" t="inlineStr">
+        <is>
+          <t>Micro-milled creamy white pepper powder for luxury banquet seasoning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-005</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>Salem Golden Turmeric Powder</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D9" s="39" t="inlineStr">
+        <is>
+          <t>09103030</t>
+        </is>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>260</v>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>40kg Triple-Lined Bags</t>
+        </is>
+      </c>
+      <c r="G9" s="38" t="inlineStr">
+        <is>
+          <t>High curcumin Salem native rhizome ground. Zero lead chromate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-006</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>Scarlet Kashmiri Chilly (Whole Stemless)</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>09042219</t>
+        </is>
+      </c>
+      <c r="E10" s="44" t="n">
+        <v>580</v>
+      </c>
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G10" s="42" t="inlineStr">
+        <is>
+          <t>Sun-dried wrinkled crimson Kashmiri chillies for royal tandoor &amp; biryani color.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-007</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>Pure Kashmiri Chilli Powder</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D11" s="39" t="inlineStr">
+        <is>
+          <t>09042211</t>
+        </is>
+      </c>
+      <c r="E11" s="40" t="n">
+        <v>620</v>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>Cold-pulverized bright scarlet chilli powder. Intense natural colour extraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-008</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>Guntur S17 Whole Stemless Red Chilli</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>09042110</t>
+        </is>
+      </c>
+      <c r="E12" s="44" t="n">
+        <v>320</v>
+      </c>
+      <c r="F12" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G12" s="42" t="inlineStr">
+        <is>
+          <t>High-pungency fiery Guntur S17 chillies for bold South Indian curries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-009</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>Guntur Spicy Red Chilli Powder</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D13" s="39" t="inlineStr">
+        <is>
+          <t>09042211</t>
+        </is>
+      </c>
+      <c r="E13" s="40" t="n">
+        <v>340</v>
+      </c>
+      <c r="F13" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G13" s="38" t="inlineStr">
+        <is>
+          <t>Stone-milled fiery red chilli powder for high-volume commercial kitchens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-010</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>Alleppey Green Cardamom (8mm+ Extra Bold)</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D14" s="43" t="inlineStr">
+        <is>
+          <t>09083140</t>
+        </is>
+      </c>
+      <c r="E14" s="44" t="n">
+        <v>2800</v>
+      </c>
+      <c r="F14" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G14" s="42" t="inlineStr">
+        <is>
+          <t>Hand-graded 8mm+ calibrated pods. High natural essential oils and aroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-011</t>
+        </is>
+      </c>
+      <c r="B15" s="38" t="inlineStr">
+        <is>
+          <t>Stone Milled Green Cardamom Powder</t>
+        </is>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D15" s="39" t="inlineStr">
+        <is>
+          <t>09083200</t>
+        </is>
+      </c>
+      <c r="E15" s="40" t="n">
+        <v>2950</v>
+      </c>
+      <c r="F15" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G15" s="38" t="inlineStr">
+        <is>
+          <t>Whole-pod stone milled green cardamom powder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-012</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>Large Hill Black Cardamom (Badi Elaichi)</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>09083110</t>
+        </is>
+      </c>
+      <c r="E16" s="44" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F16" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G16" s="42" t="inlineStr">
+        <is>
+          <t>Smoked sun-cured hill black cardamom pods for royal dum biryani.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-013</t>
+        </is>
+      </c>
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Bleached / Decorticated White Cardamom</t>
+        </is>
+      </c>
+      <c r="C17" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D17" s="39" t="inlineStr">
+        <is>
+          <t>09083120</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="n">
+        <v>2400</v>
+      </c>
+      <c r="F17" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G17" s="38" t="inlineStr">
+        <is>
+          <t>Delicate aromatic white cardamom for sweets and fine confectionery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-014</t>
+        </is>
+      </c>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Cochin Sun-Cured Dry Ginger (Unbleached Whole)</t>
+        </is>
+      </c>
+      <c r="C18" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>09101110</t>
+        </is>
+      </c>
+      <c r="E18" s="44" t="n">
+        <v>460</v>
+      </c>
+      <c r="F18" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>Premium Cochin whole dry ginger rhizomes with sharp gingerol pungency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-015</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>Pure Sun-Dried Sonth Ginger Powder</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D19" s="39" t="inlineStr">
+        <is>
+          <t>09101200</t>
+        </is>
+      </c>
+      <c r="E19" s="40" t="n">
+        <v>490</v>
+      </c>
+      <c r="F19" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G19" s="38" t="inlineStr">
+        <is>
+          <t>Finely ground unbleached dry ginger powder for marinades and chai blends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-016</t>
+        </is>
+      </c>
+      <c r="B20" s="42" t="inlineStr">
+        <is>
+          <t>Whole Green Coriander Seeds (Dhania Whole)</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>09092190</t>
+        </is>
+      </c>
+      <c r="E20" s="44" t="n">
+        <v>175</v>
+      </c>
+      <c r="F20" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>Sortex-cleaned whole coriander seeds for crisp citrusy aroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-017</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>Cold-Milled Coriander Powder (Dhania Powder)</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D21" s="39" t="inlineStr">
+        <is>
+          <t>09092200</t>
+        </is>
+      </c>
+      <c r="E21" s="40" t="n">
+        <v>195</v>
+      </c>
+      <c r="F21" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G21" s="38" t="inlineStr">
+        <is>
+          <t>Cold-milled fragrant coriander powder. Single-origin unadulterated aroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-018</t>
+        </is>
+      </c>
+      <c r="B22" s="42" t="inlineStr">
+        <is>
+          <t>Machine-Cleaned Cumin Seeds (Jeera Whole)</t>
+        </is>
+      </c>
+      <c r="C22" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>09093129</t>
+        </is>
+      </c>
+      <c r="E22" s="44" t="n">
+        <v>380</v>
+      </c>
+      <c r="F22" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G22" s="42" t="inlineStr">
+        <is>
+          <t>99.5% machine-cleaned whole cumin seeds with rich essential cumin oil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-019</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>Stone-Milled Jeera Cumin Powder</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>09093200</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="n">
+        <v>420</v>
+      </c>
+      <c r="F23" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G23" s="38" t="inlineStr">
+        <is>
+          <t>Aromatic ground cumin powder stone-milled from pure seed lots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-020</t>
+        </is>
+      </c>
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Imperial Shahi Jeera (Wild Mountain Caraway)</t>
+        </is>
+      </c>
+      <c r="C24" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>09096119</t>
+        </is>
+      </c>
+      <c r="E24" s="44" t="n">
+        <v>850</v>
+      </c>
+      <c r="F24" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G24" s="42" t="inlineStr">
+        <is>
+          <t>Fine needle-thin wild mountain caraway seeds for Rogan Josh &amp; royal pulao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-021</t>
+        </is>
+      </c>
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t>Zanzibar Whole Handpicked Cloves (Laung)</t>
+        </is>
+      </c>
+      <c r="C25" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D25" s="39" t="inlineStr">
+        <is>
+          <t>09071010</t>
+        </is>
+      </c>
+      <c r="E25" s="40" t="n">
+        <v>980</v>
+      </c>
+      <c r="F25" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G25" s="38" t="inlineStr">
+        <is>
+          <t>Head-on, bold, oil-rich Zanzibar whole cloves. Zero spent headless buds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-022</t>
+        </is>
+      </c>
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t>True Ceylon Cinnamon Quills (C5 Alba Pattai)</t>
+        </is>
+      </c>
+      <c r="C26" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>09061110</t>
+        </is>
+      </c>
+      <c r="E26" s="44" t="n">
+        <v>1250</v>
+      </c>
+      <c r="F26" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bundles</t>
+        </is>
+      </c>
+      <c r="G26" s="42" t="inlineStr">
+        <is>
+          <t>Delicate multi-layered thin bark quills of true Ceylon cinnamon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-023</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>High-Aroma Cassia Bark Slices (Kesia Pattai)</t>
+        </is>
+      </c>
+      <c r="C27" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D27" s="39" t="inlineStr">
+        <is>
+          <t>09061910</t>
+        </is>
+      </c>
+      <c r="E27" s="40" t="n">
+        <v>360</v>
+      </c>
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G27" s="38" t="inlineStr">
+        <is>
+          <t>Thick rolled aromatic cassia bark for robust biryani tempering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-024</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>8-Pointed Autumn Star Anise (Annachipoo)</t>
+        </is>
+      </c>
+      <c r="C28" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>09096115</t>
+        </is>
+      </c>
+      <c r="E28" s="44" t="n">
+        <v>820</v>
+      </c>
+      <c r="F28" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G28" s="42" t="inlineStr">
+        <is>
+          <t>Whole unbroken 8-pointed star anise flowers with rich anethole aroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-025</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Bold Green Fennel Seeds (Sombu / Saunf)</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D29" s="39" t="inlineStr">
+        <is>
+          <t>09096145</t>
+        </is>
+      </c>
+      <c r="E29" s="40" t="n">
+        <v>280</v>
+      </c>
+      <c r="F29" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G29" s="38" t="inlineStr">
+        <is>
+          <t>Machine-cleaned sweet plump green fennel seeds. Naturally sweet aroma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-026</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>Whole Nutmeg with Shell / Kernel (Jaifal)</t>
+        </is>
+      </c>
+      <c r="C30" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D30" s="43" t="inlineStr">
+        <is>
+          <t>09081110</t>
+        </is>
+      </c>
+      <c r="E30" s="44" t="n">
+        <v>780</v>
+      </c>
+      <c r="F30" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G30" s="42" t="inlineStr">
+        <is>
+          <t>Dense whole nutmeg nuts with intact inner volatile oil kernel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-027</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Banded Golden Mace Blades (Javantri)</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D31" s="39" t="inlineStr">
+        <is>
+          <t>09082100</t>
+        </is>
+      </c>
+      <c r="E31" s="40" t="n">
+        <v>1950</v>
+      </c>
+      <c r="F31" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G31" s="38" t="inlineStr">
+        <is>
+          <t>Vibrant golden-orange unbroken flower mace blades with spicy fragrance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-028</t>
+        </is>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
+          <t>Sun-Dried Biryani Bay Leaves (Tejpatta)</t>
+        </is>
+      </c>
+      <c r="C32" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D32" s="43" t="inlineStr">
+        <is>
+          <t>09109914</t>
+        </is>
+      </c>
+      <c r="E32" s="44" t="n">
+        <v>180</v>
+      </c>
+      <c r="F32" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G32" s="42" t="inlineStr">
+        <is>
+          <t>Fragrant whole unbroken Ceylon bay leaves for slow dum cooking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-029</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>Black Stone Flower (Kalpasi / Dagad Phool)</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D33" s="39" t="inlineStr">
+        <is>
+          <t>09109990</t>
+        </is>
+      </c>
+      <c r="E33" s="40" t="n">
+        <v>640</v>
+      </c>
+      <c r="F33" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G33" s="38" t="inlineStr">
+        <is>
+          <t>Wild-harvested black and silver stone lichen for authentic Chettinad gravies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-030</t>
+        </is>
+      </c>
+      <c r="B34" s="42" t="inlineStr">
+        <is>
+          <t>Fragrant Green Kasuri Methi (Nagauri Leaves)</t>
+        </is>
+      </c>
+      <c r="C34" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>09109915</t>
+        </is>
+      </c>
+      <c r="E34" s="44" t="n">
+        <v>340</v>
+      </c>
+      <c r="F34" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G34" s="42" t="inlineStr">
+        <is>
+          <t>Shadow-dried vibrant green fenugreek leaves. Zero sand or stalk debris.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-031</t>
+        </is>
+      </c>
+      <c r="B35" s="38" t="inlineStr">
+        <is>
+          <t>Selected Whole Fenugreek Seeds (Methi)</t>
+        </is>
+      </c>
+      <c r="C35" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D35" s="39" t="inlineStr">
+        <is>
+          <t>09109912</t>
+        </is>
+      </c>
+      <c r="E35" s="40" t="n">
+        <v>135</v>
+      </c>
+      <c r="F35" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G35" s="38" t="inlineStr">
+        <is>
+          <t>Bold sortex-cleaned whole fenugreek seeds for sambar and pickle masalas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-032</t>
+        </is>
+      </c>
+      <c r="B36" s="42" t="inlineStr">
+        <is>
+          <t>Bold Black Mustard Seeds (Kadugu / Rai)</t>
+        </is>
+      </c>
+      <c r="C36" s="43" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>09109911</t>
+        </is>
+      </c>
+      <c r="E36" s="44" t="n">
+        <v>125</v>
+      </c>
+      <c r="F36" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G36" s="42" t="inlineStr">
+        <is>
+          <t>Selected bold black mustard seeds with high popping oil vitality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-033</t>
+        </is>
+      </c>
+      <c r="B37" s="38" t="inlineStr">
+        <is>
+          <t>Pure Black Nigella Seeds (Kalonji)</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>Single-Origin Spices</t>
+        </is>
+      </c>
+      <c r="D37" s="39" t="inlineStr">
+        <is>
+          <t>09096149</t>
+        </is>
+      </c>
+      <c r="E37" s="40" t="n">
+        <v>360</v>
+      </c>
+      <c r="F37" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G37" s="38" t="inlineStr">
+        <is>
+          <t>Triple-cleaned black nigella seeds for naan bread crusts and tempering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="41" t="inlineStr">
+        <is>
+          <t>KTA-BL-001</t>
+        </is>
+      </c>
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>Royal Chef Garam Masala (Whole Spice Blend)</t>
+        </is>
+      </c>
+      <c r="C38" s="43" t="inlineStr">
+        <is>
+          <t>Culinary Blends</t>
+        </is>
+      </c>
+      <c r="D38" s="43" t="inlineStr">
+        <is>
+          <t>09109100</t>
+        </is>
+      </c>
+      <c r="E38" s="44" t="n">
+        <v>880</v>
+      </c>
+      <c r="F38" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G38" s="42" t="inlineStr">
+        <is>
+          <t>Master chef artisanal blend of 14 whole roasted single-origin spices. Zero fillers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="37" t="inlineStr">
+        <is>
+          <t>KTA-BL-002</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="inlineStr">
+        <is>
+          <t>Royal Dum Biryani Masala (Pristine Blend)</t>
+        </is>
+      </c>
+      <c r="C39" s="39" t="inlineStr">
+        <is>
+          <t>Culinary Blends</t>
+        </is>
+      </c>
+      <c r="D39" s="39" t="inlineStr">
+        <is>
+          <t>09109100</t>
+        </is>
+      </c>
+      <c r="E39" s="40" t="n">
+        <v>940</v>
+      </c>
+      <c r="F39" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G39" s="38" t="inlineStr">
+        <is>
+          <t>Heritage aromatic spice blend curated for luxury hotel biryanis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="41" t="inlineStr">
+        <is>
+          <t>KTA-SP-034</t>
+        </is>
+      </c>
+      <c r="B40" s="42" t="inlineStr">
+        <is>
+          <t>Sun-Cured Black Dry Lemon (Loomi Whole)</t>
+        </is>
+      </c>
+      <c r="C40" s="43" t="inlineStr">
+        <is>
+          <t>Specialty Botanicals</t>
+        </is>
+      </c>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>08055000</t>
+        </is>
+      </c>
+      <c r="E40" s="44" t="n">
+        <v>520</v>
+      </c>
+      <c r="F40" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G40" s="42" t="inlineStr">
+        <is>
+          <t>Traditional sun-dried black lime for Arabian mandi and broths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="37" t="inlineStr">
+        <is>
+          <t>KTA-SP-035</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="inlineStr">
+        <is>
+          <t>Super Mongra Kashmiri Saffron (Grade A1)</t>
+        </is>
+      </c>
+      <c r="C41" s="39" t="inlineStr">
+        <is>
+          <t>Specialty Botanicals</t>
+        </is>
+      </c>
+      <c r="D41" s="39" t="inlineStr">
+        <is>
+          <t>09102010</t>
+        </is>
+      </c>
+      <c r="E41" s="40" t="n">
+        <v>260000</v>
+      </c>
+      <c r="F41" s="38" t="inlineStr">
+        <is>
+          <t>1kg Master Packaging</t>
+        </is>
+      </c>
+      <c r="G41" s="38" t="inlineStr">
+        <is>
+          <t>Pristine deep crimson saffron stigmas without yellow style adulteration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-001</t>
+        </is>
+      </c>
+      <c r="B42" s="42" t="inlineStr">
+        <is>
+          <t>California Bold Whole Almonds (Badam 18/20)</t>
+        </is>
+      </c>
+      <c r="C42" s="43" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D42" s="43" t="inlineStr">
+        <is>
+          <t>08021200</t>
+        </is>
+      </c>
+      <c r="E42" s="44" t="n">
+        <v>780</v>
+      </c>
+      <c r="F42" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G42" s="42" t="inlineStr">
+        <is>
+          <t>Jumbo size 18/20 count premium raw California almonds. Crisp sweet bite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-002</t>
+        </is>
+      </c>
+      <c r="B43" s="38" t="inlineStr">
+        <is>
+          <t>W320 First Quality Jumbo White Cashews (Kaju)</t>
+        </is>
+      </c>
+      <c r="C43" s="39" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D43" s="39" t="inlineStr">
+        <is>
+          <t>08013100</t>
+        </is>
+      </c>
+      <c r="E43" s="40" t="n">
+        <v>860</v>
+      </c>
+      <c r="F43" s="38" t="inlineStr">
+        <is>
+          <t>50kg Master Jute Bags</t>
+        </is>
+      </c>
+      <c r="G43" s="38" t="inlineStr">
+        <is>
+          <t>Whole unblemished W320 grade white cashew nuts. Creamy rich texture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-003</t>
+        </is>
+      </c>
+      <c r="B44" s="42" t="inlineStr">
+        <is>
+          <t>California Roasted &amp; Salted Pistachios (Pista)</t>
+        </is>
+      </c>
+      <c r="C44" s="43" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D44" s="43" t="inlineStr">
+        <is>
+          <t>08025100</t>
+        </is>
+      </c>
+      <c r="E44" s="44" t="n">
+        <v>1150</v>
+      </c>
+      <c r="F44" s="42" t="inlineStr">
+        <is>
+          <t>10kg Master Cartons</t>
+        </is>
+      </c>
+      <c r="G44" s="42" t="inlineStr">
+        <is>
+          <t>Naturally opened jumbo roasted pistachios with light sea salt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-004</t>
+        </is>
+      </c>
+      <c r="B45" s="38" t="inlineStr">
+        <is>
+          <t>California Light Quarter Walnut Kernels (Akhrot)</t>
+        </is>
+      </c>
+      <c r="C45" s="39" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D45" s="39" t="inlineStr">
+        <is>
+          <t>08023200</t>
+        </is>
+      </c>
+      <c r="E45" s="40" t="n">
+        <v>1180</v>
+      </c>
+      <c r="F45" s="38" t="inlineStr">
+        <is>
+          <t>10kg Master Cartons</t>
+        </is>
+      </c>
+      <c r="G45" s="38" t="inlineStr">
+        <is>
+          <t>Fresh crisp light amber walnut halves &amp; quarters. Zero rancidity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-005</t>
+        </is>
+      </c>
+      <c r="B46" s="42" t="inlineStr">
+        <is>
+          <t>Golden Long Seedless Raisins (Kismiss)</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>08062010</t>
+        </is>
+      </c>
+      <c r="E46" s="44" t="n">
+        <v>340</v>
+      </c>
+      <c r="F46" s="42" t="inlineStr">
+        <is>
+          <t>15kg Master Cartons</t>
+        </is>
+      </c>
+      <c r="G46" s="42" t="inlineStr">
+        <is>
+          <t>Plump sun-dried green-gold seedless raisins for biryani and desserts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-006</t>
+        </is>
+      </c>
+      <c r="B47" s="38" t="inlineStr">
+        <is>
+          <t>Selected Black Seedless Raisins (Black Kismiss)</t>
+        </is>
+      </c>
+      <c r="C47" s="39" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D47" s="39" t="inlineStr">
+        <is>
+          <t>08062010</t>
+        </is>
+      </c>
+      <c r="E47" s="40" t="n">
+        <v>380</v>
+      </c>
+      <c r="F47" s="38" t="inlineStr">
+        <is>
+          <t>15kg Master Cartons</t>
+        </is>
+      </c>
+      <c r="G47" s="38" t="inlineStr">
+        <is>
+          <t>Plump nutrient-dense black seedless raisins for baking and confectionery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-007</t>
+        </is>
+      </c>
+      <c r="B48" s="42" t="inlineStr">
+        <is>
+          <t>Groundnut Seeds (Selected Grade Raw Peanut)</t>
+        </is>
+      </c>
+      <c r="C48" s="43" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>12024190</t>
+        </is>
+      </c>
+      <c r="E48" s="44" t="n">
+        <v>180</v>
+      </c>
+      <c r="F48" s="42" t="inlineStr">
+        <is>
+          <t>50kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G48" s="42" t="inlineStr">
+        <is>
+          <t>Selected bold raw peanut kernels with high natural oil content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-008</t>
+        </is>
+      </c>
+      <c r="B49" s="38" t="inlineStr">
+        <is>
+          <t>Dry Roasted Peanuts (Golden Crunch Husked)</t>
+        </is>
+      </c>
+      <c r="C49" s="39" t="inlineStr">
+        <is>
+          <t>Dry Fruits &amp; Nuts</t>
+        </is>
+      </c>
+      <c r="D49" s="39" t="inlineStr">
+        <is>
+          <t>20081111</t>
+        </is>
+      </c>
+      <c r="E49" s="40" t="n">
+        <v>220</v>
+      </c>
+      <c r="F49" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G49" s="38" t="inlineStr">
+        <is>
+          <t>Uniformly dry roasted and husked golden crunchy peanuts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-009</t>
+        </is>
+      </c>
+      <c r="B50" s="42" t="inlineStr">
+        <is>
+          <t>Triple-Cleaned White Sesame Seeds (White Ellu)</t>
+        </is>
+      </c>
+      <c r="C50" s="43" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr">
+        <is>
+          <t>12074090</t>
+        </is>
+      </c>
+      <c r="E50" s="44" t="n">
+        <v>260</v>
+      </c>
+      <c r="F50" s="42" t="inlineStr">
+        <is>
+          <t>40kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G50" s="42" t="inlineStr">
+        <is>
+          <t>99.9% machine-cleaned triple sortex hulled white sesame seeds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-010</t>
+        </is>
+      </c>
+      <c r="B51" s="38" t="inlineStr">
+        <is>
+          <t>Sweet Basil Seeds (Sabja / Falooda Seeds)</t>
+        </is>
+      </c>
+      <c r="C51" s="39" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D51" s="39" t="inlineStr">
+        <is>
+          <t>12119094</t>
+        </is>
+      </c>
+      <c r="E51" s="40" t="n">
+        <v>380</v>
+      </c>
+      <c r="F51" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G51" s="38" t="inlineStr">
+        <is>
+          <t>High-expansion whole sweet basil seeds for falooda and cooling drinks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-011</t>
+        </is>
+      </c>
+      <c r="B52" s="42" t="inlineStr">
+        <is>
+          <t>Premium Whole Chia Seeds (Salvia Hispanica)</t>
+        </is>
+      </c>
+      <c r="C52" s="43" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>12149000</t>
+        </is>
+      </c>
+      <c r="E52" s="44" t="n">
+        <v>420</v>
+      </c>
+      <c r="F52" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G52" s="42" t="inlineStr">
+        <is>
+          <t>Triple-cleaned whole black &amp; white chia seeds rich in soluble fiber.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-012</t>
+        </is>
+      </c>
+      <c r="B53" s="38" t="inlineStr">
+        <is>
+          <t>Raw Hulled Pumpkin Seeds (Pepitas / Kaddu Beej)</t>
+        </is>
+      </c>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D53" s="39" t="inlineStr">
+        <is>
+          <t>12099990</t>
+        </is>
+      </c>
+      <c r="E53" s="40" t="n">
+        <v>490</v>
+      </c>
+      <c r="F53" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G53" s="38" t="inlineStr">
+        <is>
+          <t>Vibrant green hulled raw pumpkin seeds (AA Grade) for bakery and salads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-013</t>
+        </is>
+      </c>
+      <c r="B54" s="42" t="inlineStr">
+        <is>
+          <t>Raw Hulled Sunflower Seeds (Surajmukhi Beej)</t>
+        </is>
+      </c>
+      <c r="C54" s="43" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D54" s="43" t="inlineStr">
+        <is>
+          <t>12060090</t>
+        </is>
+      </c>
+      <c r="E54" s="44" t="n">
+        <v>320</v>
+      </c>
+      <c r="F54" s="42" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G54" s="42" t="inlineStr">
+        <is>
+          <t>Jumbo kernel hulled sunflower seeds for granolas and breads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="37" t="inlineStr">
+        <is>
+          <t>KTA-DF-014</t>
+        </is>
+      </c>
+      <c r="B55" s="38" t="inlineStr">
+        <is>
+          <t>Peeled Watermelon Seeds (Magaz / Tarbooj Beej)</t>
+        </is>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>Edible Seeds</t>
+        </is>
+      </c>
+      <c r="D55" s="39" t="inlineStr">
+        <is>
+          <t>12079990</t>
+        </is>
+      </c>
+      <c r="E55" s="40" t="n">
+        <v>540</v>
+      </c>
+      <c r="F55" s="38" t="inlineStr">
+        <is>
+          <t>25kg Master Bags</t>
+        </is>
+      </c>
+      <c r="G55" s="38" t="inlineStr">
+        <is>
+          <t>Clean white shelled watermelon kernels for rich Mughlai curries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="41" t="inlineStr">
+        <is>
+          <t>KTA-DF-015</t>
+        </is>
+      </c>
+      <c r="B56" s="42" t="inlineStr">
+        <is>
+          <t>Culinary Dried Damascena Rose Petals (Gulab)</t>
+        </is>
+      </c>
+      <c r="C56" s="43" t="inlineStr">
+        <is>
+          <t>Specialty Botanicals</t>
+        </is>
+      </c>
+      <c r="D56" s="43" t="inlineStr">
+        <is>
+          <t>12119029</t>
+        </is>
+      </c>
+      <c r="E56" s="44" t="n">
+        <v>680</v>
+      </c>
+      <c r="F56" s="42" t="inlineStr">
+        <is>
+          <t>10kg Master Cartons</t>
+        </is>
+      </c>
+      <c r="G56" s="42" t="inlineStr">
+        <is>
+          <t>Naturally shade-dried intensely fragrant Damascena rose petals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="37" t="inlineStr">
+        <is>
+          <t>KTA-WS-001</t>
+        </is>
+      </c>
+      <c r="B57" s="38" t="inlineStr">
+        <is>
+          <t>Green Ginger (Raw Fresh Jumbo Rhizomes)</t>
+        </is>
+      </c>
+      <c r="C57" s="39" t="inlineStr">
+        <is>
+          <t>Wholesale &amp; Fresh</t>
+        </is>
+      </c>
+      <c r="D57" s="39" t="inlineStr">
+        <is>
+          <t>09101110</t>
+        </is>
+      </c>
+      <c r="E57" s="40" t="n">
+        <v>120</v>
+      </c>
+      <c r="F57" s="38" t="inlineStr">
+        <is>
+          <t>40kg Master Crates (500kg+ MOQ)</t>
+        </is>
+      </c>
+      <c r="G57" s="38" t="inlineStr">
+        <is>
+          <t>Raw fresh plump farm-direct ginger rhizomes. High juice extraction yield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="41" t="inlineStr">
+        <is>
+          <t>KTA-WS-002</t>
+        </is>
+      </c>
+      <c r="B58" s="42" t="inlineStr">
+        <is>
+          <t>Pepper Husk &amp; Pepper Husk (S) Mesh Cuts</t>
+        </is>
+      </c>
+      <c r="C58" s="43" t="inlineStr">
+        <is>
+          <t>Wholesale Extraction</t>
+        </is>
+      </c>
+      <c r="D58" s="43" t="inlineStr">
+        <is>
+          <t>09041140</t>
+        </is>
+      </c>
+      <c r="E58" s="44" t="n">
+        <v>140</v>
+      </c>
+      <c r="F58" s="42" t="inlineStr">
+        <is>
+          <t>50kg Bags (500kg+ MOQ)</t>
+        </is>
+      </c>
+      <c r="G58" s="42" t="inlineStr">
+        <is>
+          <t>Clean sieved black pepper outer husk. High piperine resin for oleoresin extraction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="37" t="inlineStr">
+        <is>
+          <t>KTA-WS-003</t>
+        </is>
+      </c>
+      <c r="B59" s="38" t="inlineStr">
+        <is>
+          <t>Black Pepper Lite Berries &amp; Pinheads</t>
+        </is>
+      </c>
+      <c r="C59" s="39" t="inlineStr">
+        <is>
+          <t>Wholesale Extraction</t>
+        </is>
+      </c>
+      <c r="D59" s="39" t="inlineStr">
+        <is>
+          <t>09041140</t>
+        </is>
+      </c>
+      <c r="E59" s="40" t="n">
+        <v>280</v>
+      </c>
+      <c r="F59" s="38" t="inlineStr">
+        <is>
+          <t>50kg Bags (500kg+ MOQ)</t>
+        </is>
+      </c>
+      <c r="G59" s="38" t="inlineStr">
+        <is>
+          <t>High oleoresin concentration lightweight berries and whole pinheads for extraction units.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>